<commit_message>
sort of rag is build
</commit_message>
<xml_diff>
--- a/data/placement.xlsx
+++ b/data/placement.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NEWChatbotADCET\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F77116-38BC-40CD-B7AB-DFCA9A9DB271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52232875-1F71-4C00-953D-FF417A950458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{74B4B548-AF3E-4B86-BB54-426AD5125710}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{74B4B548-AF3E-4B86-BB54-426AD5125710}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="cutoff" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="293">
   <si>
     <t>Company Name</t>
   </si>
@@ -845,13 +846,82 @@
   </si>
   <si>
     <t>Acadamic Year:- 2023-24</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Course</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>G(General)</t>
+  </si>
+  <si>
+    <t>L(Ledies)</t>
+  </si>
+  <si>
+    <t>VJ</t>
+  </si>
+  <si>
+    <t>Merit No</t>
+  </si>
+  <si>
+    <t>Merit Marks</t>
+  </si>
+  <si>
+    <t>NT-1</t>
+  </si>
+  <si>
+    <t>NT-2</t>
+  </si>
+  <si>
+    <t>NT-3</t>
+  </si>
+  <si>
+    <t>OBC</t>
+  </si>
+  <si>
+    <t>SEBC</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>DEF</t>
+  </si>
+  <si>
+    <t>TFWS</t>
+  </si>
+  <si>
+    <t>EWS</t>
+  </si>
+  <si>
+    <t>RAI</t>
+  </si>
+  <si>
+    <t>ELEC</t>
+  </si>
+  <si>
+    <t>CS IOT</t>
+  </si>
+  <si>
+    <t>CIVIL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -921,6 +991,31 @@
       <name val="Book Antiqua"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="Book Antiqua"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="Book Antiqua"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Book Antiqua"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Book Antiqua"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1348,7 +1443,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1470,108 +1565,121 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1896,11 +2004,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="73" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
     </row>
     <row r="2" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -2673,11 +2781,11 @@
       </c>
     </row>
     <row r="72" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="41" t="s">
+      <c r="A72" s="73" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="42"/>
-      <c r="C72" s="42"/>
+      <c r="B72" s="74"/>
+      <c r="C72" s="74"/>
     </row>
     <row r="73" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="30" t="s">
@@ -3483,11 +3591,11 @@
       </c>
     </row>
     <row r="146" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A146" s="41" t="s">
+      <c r="A146" s="73" t="s">
         <v>177</v>
       </c>
-      <c r="B146" s="42"/>
-      <c r="C146" s="42"/>
+      <c r="B146" s="74"/>
+      <c r="C146" s="74"/>
     </row>
     <row r="147" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="20" t="s">
@@ -4418,550 +4526,2161 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="41" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="42" t="s">
         <v>249</v>
       </c>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
     </row>
     <row r="2" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="45"/>
-      <c r="B2" s="46" t="s">
+      <c r="A2" s="43"/>
+      <c r="B2" s="44" t="s">
         <v>250</v>
       </c>
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="44" t="s">
         <v>252</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="44" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="46" t="s">
         <v>254</v>
       </c>
-      <c r="B3" s="49">
+      <c r="B3" s="47">
         <v>96</v>
       </c>
-      <c r="C3" s="50">
+      <c r="C3" s="48">
         <v>122</v>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="48">
         <v>5</v>
       </c>
-      <c r="E3" s="50">
+      <c r="E3" s="48">
         <v>8.5</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="49" t="s">
         <v>255</v>
       </c>
-      <c r="B4" s="52">
+      <c r="B4" s="50">
         <v>34</v>
       </c>
-      <c r="C4" s="53">
+      <c r="C4" s="51">
         <v>37</v>
       </c>
-      <c r="D4" s="53">
+      <c r="D4" s="51">
         <v>5</v>
       </c>
-      <c r="E4" s="53">
+      <c r="E4" s="51">
         <v>6.5</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="B5" s="52">
+      <c r="B5" s="50">
         <v>153</v>
       </c>
-      <c r="C5" s="53">
+      <c r="C5" s="51">
         <v>171</v>
       </c>
-      <c r="D5" s="53">
+      <c r="D5" s="51">
         <v>5</v>
       </c>
-      <c r="E5" s="53">
+      <c r="E5" s="51">
         <v>6.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="49" t="s">
         <v>257</v>
       </c>
-      <c r="B6" s="52">
+      <c r="B6" s="50">
         <v>145</v>
       </c>
-      <c r="C6" s="53">
+      <c r="C6" s="51">
         <v>120</v>
       </c>
-      <c r="D6" s="53">
+      <c r="D6" s="51">
         <v>5.2</v>
       </c>
-      <c r="E6" s="53">
+      <c r="E6" s="51">
         <v>12.34</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="49" t="s">
         <v>258</v>
       </c>
-      <c r="B7" s="52">
+      <c r="B7" s="50">
         <v>69</v>
       </c>
-      <c r="C7" s="53">
+      <c r="C7" s="51">
         <v>41</v>
       </c>
-      <c r="D7" s="53">
+      <c r="D7" s="51">
         <v>5.2</v>
       </c>
-      <c r="E7" s="53">
+      <c r="E7" s="51">
         <v>8.67</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="49" t="s">
         <v>259</v>
       </c>
-      <c r="B8" s="52">
+      <c r="B8" s="50">
         <v>73</v>
       </c>
-      <c r="C8" s="53">
+      <c r="C8" s="51">
         <v>43</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="51">
         <v>5.2</v>
       </c>
-      <c r="E8" s="53">
+      <c r="E8" s="51">
         <v>7.5</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="51" t="s">
+      <c r="A9" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="B9" s="52">
+      <c r="B9" s="50">
         <v>48</v>
       </c>
-      <c r="C9" s="53">
+      <c r="C9" s="51">
         <v>33</v>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="51">
         <v>4.5999999999999996</v>
       </c>
-      <c r="E9" s="53">
+      <c r="E9" s="51">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="51" t="s">
+      <c r="A10" s="49" t="s">
         <v>261</v>
       </c>
-      <c r="B10" s="52">
+      <c r="B10" s="50">
         <v>8</v>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="51">
         <v>21</v>
       </c>
-      <c r="D10" s="53">
-        <v>4</v>
-      </c>
-      <c r="E10" s="53">
+      <c r="D10" s="51">
+        <v>4</v>
+      </c>
+      <c r="E10" s="51">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="51" t="s">
+      <c r="A11" s="49" t="s">
         <v>262</v>
       </c>
-      <c r="B11" s="51"/>
-      <c r="C11" s="66" t="s">
+      <c r="B11" s="49"/>
+      <c r="C11" s="61" t="s">
         <v>263</v>
       </c>
-      <c r="D11" s="67"/>
-      <c r="E11" s="68"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="63"/>
     </row>
     <row r="12" spans="1:5" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="52" t="s">
         <v>264</v>
       </c>
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="64" t="s">
         <v>265</v>
       </c>
-      <c r="C12" s="56"/>
-      <c r="D12" s="56"/>
-      <c r="E12" s="57"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="66"/>
     </row>
     <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="58"/>
-      <c r="B13" s="44" t="s">
+      <c r="A13" s="53"/>
+      <c r="B13" s="42" t="s">
         <v>266</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
     </row>
     <row r="14" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="58"/>
-      <c r="B14" s="46" t="s">
+      <c r="A14" s="53"/>
+      <c r="B14" s="44" t="s">
         <v>250</v>
       </c>
-      <c r="C14" s="47" t="s">
+      <c r="C14" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="44" t="s">
         <v>252</v>
       </c>
-      <c r="E14" s="46" t="s">
+      <c r="E14" s="44" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="46" t="s">
         <v>254</v>
       </c>
-      <c r="B15" s="59">
+      <c r="B15" s="54">
         <v>87</v>
       </c>
-      <c r="C15" s="50">
+      <c r="C15" s="48">
         <v>132</v>
       </c>
-      <c r="D15" s="50">
+      <c r="D15" s="48">
         <v>4.7</v>
       </c>
-      <c r="E15" s="60">
+      <c r="E15" s="55">
         <v>6.5</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="51" t="s">
+      <c r="A16" s="49" t="s">
         <v>255</v>
       </c>
-      <c r="B16" s="61">
+      <c r="B16" s="56">
         <v>70</v>
       </c>
-      <c r="C16" s="53">
+      <c r="C16" s="51">
         <v>30</v>
       </c>
-      <c r="D16" s="53">
+      <c r="D16" s="51">
         <v>4.8</v>
       </c>
-      <c r="E16" s="62">
+      <c r="E16" s="57">
         <v>7.5</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="51" t="s">
+      <c r="A17" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="B17" s="61">
+      <c r="B17" s="56">
         <v>146</v>
       </c>
-      <c r="C17" s="53">
+      <c r="C17" s="51">
         <v>127</v>
       </c>
-      <c r="D17" s="53">
+      <c r="D17" s="51">
         <v>5.2</v>
       </c>
-      <c r="E17" s="62">
+      <c r="E17" s="57">
         <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="51" t="s">
+      <c r="A18" s="49" t="s">
         <v>257</v>
       </c>
-      <c r="B18" s="61">
+      <c r="B18" s="56">
         <v>131</v>
       </c>
-      <c r="C18" s="53">
+      <c r="C18" s="51">
         <v>90</v>
       </c>
-      <c r="D18" s="53">
+      <c r="D18" s="51">
         <v>5.2</v>
       </c>
-      <c r="E18" s="62">
+      <c r="E18" s="57">
         <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="51" t="s">
+      <c r="A19" s="49" t="s">
         <v>258</v>
       </c>
-      <c r="B19" s="61">
+      <c r="B19" s="56">
         <v>62</v>
       </c>
-      <c r="C19" s="53">
+      <c r="C19" s="51">
         <v>40</v>
       </c>
-      <c r="D19" s="53">
+      <c r="D19" s="51">
         <v>5.2</v>
       </c>
-      <c r="E19" s="62">
+      <c r="E19" s="57">
         <v>7.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="51" t="s">
+      <c r="A20" s="49" t="s">
         <v>259</v>
       </c>
-      <c r="B20" s="61">
+      <c r="B20" s="56">
         <v>70</v>
       </c>
-      <c r="C20" s="53">
+      <c r="C20" s="51">
         <v>47</v>
       </c>
-      <c r="D20" s="53">
+      <c r="D20" s="51">
         <v>5.2</v>
       </c>
-      <c r="E20" s="62">
+      <c r="E20" s="57">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="51" t="s">
+      <c r="A21" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="B21" s="61">
+      <c r="B21" s="56">
         <v>33</v>
       </c>
-      <c r="C21" s="53">
+      <c r="C21" s="51">
         <v>28</v>
       </c>
-      <c r="D21" s="53">
+      <c r="D21" s="51">
         <v>4.5999999999999996</v>
       </c>
-      <c r="E21" s="62">
+      <c r="E21" s="57">
         <v>4.5</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="51" t="s">
+      <c r="A22" s="49" t="s">
         <v>261</v>
       </c>
-      <c r="B22" s="61">
+      <c r="B22" s="56">
         <v>21</v>
       </c>
-      <c r="C22" s="53">
+      <c r="C22" s="51">
         <v>17</v>
       </c>
-      <c r="D22" s="53">
+      <c r="D22" s="51">
         <v>3.5</v>
       </c>
-      <c r="E22" s="62">
+      <c r="E22" s="57">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="51" t="s">
+      <c r="A23" s="49" t="s">
         <v>262</v>
       </c>
-      <c r="B23" s="63">
+      <c r="B23" s="58">
         <v>620</v>
       </c>
-      <c r="C23" s="66" t="s">
+      <c r="C23" s="61" t="s">
         <v>267</v>
       </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="68"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="63"/>
     </row>
     <row r="24" spans="1:5" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="52" t="s">
         <v>264</v>
       </c>
-      <c r="B24" s="72" t="s">
+      <c r="B24" s="67" t="s">
         <v>268</v>
       </c>
-      <c r="C24" s="73"/>
-      <c r="D24" s="73"/>
-      <c r="E24" s="74"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="69"/>
     </row>
     <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="58"/>
-      <c r="B25" s="44" t="s">
+      <c r="A25" s="53"/>
+      <c r="B25" s="42" t="s">
         <v>269</v>
       </c>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="64"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="59"/>
     </row>
     <row r="26" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="58"/>
-      <c r="B26" s="46" t="s">
+      <c r="A26" s="53"/>
+      <c r="B26" s="44" t="s">
         <v>250</v>
       </c>
-      <c r="C26" s="47" t="s">
+      <c r="C26" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="D26" s="44" t="s">
         <v>252</v>
       </c>
-      <c r="E26" s="65" t="s">
+      <c r="E26" s="60" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="48" t="s">
+      <c r="A27" s="46" t="s">
         <v>254</v>
       </c>
-      <c r="B27" s="59">
+      <c r="B27" s="54">
         <v>112</v>
       </c>
-      <c r="C27" s="50">
+      <c r="C27" s="48">
         <v>105</v>
       </c>
-      <c r="D27" s="50">
+      <c r="D27" s="48">
         <v>4.5</v>
       </c>
-      <c r="E27" s="60">
+      <c r="E27" s="55">
         <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="51" t="s">
+      <c r="A28" s="49" t="s">
         <v>255</v>
       </c>
-      <c r="B28" s="61">
+      <c r="B28" s="56">
         <v>73</v>
       </c>
-      <c r="C28" s="53">
+      <c r="C28" s="51">
         <v>99</v>
       </c>
-      <c r="D28" s="53">
+      <c r="D28" s="51">
         <v>4.5</v>
       </c>
-      <c r="E28" s="62">
+      <c r="E28" s="57">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="51" t="s">
+      <c r="A29" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="B29" s="61">
+      <c r="B29" s="56">
         <v>145</v>
       </c>
-      <c r="C29" s="53">
+      <c r="C29" s="51">
         <v>117</v>
       </c>
-      <c r="D29" s="53">
+      <c r="D29" s="51">
         <v>4.8</v>
       </c>
-      <c r="E29" s="62">
+      <c r="E29" s="57">
         <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="51" t="s">
+      <c r="A30" s="49" t="s">
         <v>257</v>
       </c>
-      <c r="B30" s="61">
+      <c r="B30" s="56">
         <v>153</v>
       </c>
-      <c r="C30" s="53">
+      <c r="C30" s="51">
         <v>142</v>
       </c>
-      <c r="D30" s="53">
+      <c r="D30" s="51">
         <v>5</v>
       </c>
-      <c r="E30" s="62">
+      <c r="E30" s="57">
         <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="51" t="s">
+      <c r="A31" s="49" t="s">
         <v>258</v>
       </c>
-      <c r="B31" s="61"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="62"/>
+      <c r="B31" s="56"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="51"/>
+      <c r="E31" s="57"/>
     </row>
     <row r="32" spans="1:5" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="51" t="s">
+      <c r="A32" s="49" t="s">
         <v>259</v>
       </c>
-      <c r="B32" s="61"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="62"/>
+      <c r="B32" s="56"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="57"/>
     </row>
     <row r="33" spans="1:5" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="51" t="s">
+      <c r="A33" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="B33" s="61">
+      <c r="B33" s="56">
         <v>55</v>
       </c>
-      <c r="C33" s="53">
+      <c r="C33" s="51">
         <v>55</v>
       </c>
-      <c r="D33" s="53">
+      <c r="D33" s="51">
         <v>4.3</v>
       </c>
-      <c r="E33" s="62">
+      <c r="E33" s="57">
         <v>5.5</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="51" t="s">
+      <c r="A34" s="49" t="s">
         <v>261</v>
       </c>
-      <c r="B34" s="61">
+      <c r="B34" s="56">
         <v>40</v>
       </c>
-      <c r="C34" s="53">
+      <c r="C34" s="51">
         <v>36</v>
       </c>
-      <c r="D34" s="53">
+      <c r="D34" s="51">
         <v>3.8</v>
       </c>
-      <c r="E34" s="62">
+      <c r="E34" s="57">
         <v>4.5</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="51" t="s">
+      <c r="A35" s="49" t="s">
         <v>262</v>
       </c>
-      <c r="B35" s="63">
+      <c r="B35" s="58">
         <v>578</v>
       </c>
-      <c r="C35" s="66">
+      <c r="C35" s="61">
         <v>554</v>
       </c>
-      <c r="D35" s="67"/>
-      <c r="E35" s="68"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="63"/>
     </row>
     <row r="36" spans="1:5" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="54" t="s">
+      <c r="A36" s="52" t="s">
         <v>264</v>
       </c>
-      <c r="B36" s="71">
+      <c r="B36" s="70">
         <v>82</v>
       </c>
-      <c r="C36" s="69"/>
-      <c r="D36" s="69"/>
-      <c r="E36" s="70"/>
+      <c r="C36" s="71"/>
+      <c r="D36" s="71"/>
+      <c r="E36" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B36:E36"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="B36:E36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18823D42-D610-45FB-910C-BB41AA383E29}">
+  <dimension ref="A1:Z20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="12.77734375" customWidth="1"/>
+    <col min="3" max="3" width="7" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="79"/>
+      <c r="B1" s="79" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1" s="79" t="s">
+        <v>275</v>
+      </c>
+      <c r="D1" s="79" t="s">
+        <v>275</v>
+      </c>
+      <c r="E1" s="79" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1" s="79" t="s">
+        <v>278</v>
+      </c>
+      <c r="G1" s="79" t="s">
+        <v>279</v>
+      </c>
+      <c r="H1" s="79" t="s">
+        <v>279</v>
+      </c>
+      <c r="I1" s="79" t="s">
+        <v>280</v>
+      </c>
+      <c r="J1" s="79" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="79" t="s">
+        <v>281</v>
+      </c>
+      <c r="L1" s="79" t="s">
+        <v>281</v>
+      </c>
+      <c r="M1" s="79" t="s">
+        <v>282</v>
+      </c>
+      <c r="N1" s="79" t="s">
+        <v>282</v>
+      </c>
+      <c r="O1" s="79" t="s">
+        <v>283</v>
+      </c>
+      <c r="P1" s="79" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q1" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="R1" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="S1" s="79" t="s">
+        <v>285</v>
+      </c>
+      <c r="T1" s="79" t="s">
+        <v>285</v>
+      </c>
+      <c r="U1" s="79" t="s">
+        <v>286</v>
+      </c>
+      <c r="V1" s="79" t="s">
+        <v>286</v>
+      </c>
+      <c r="W1" s="79" t="s">
+        <v>287</v>
+      </c>
+      <c r="X1" s="79" t="s">
+        <v>287</v>
+      </c>
+      <c r="Y1" s="79" t="s">
+        <v>288</v>
+      </c>
+      <c r="Z1" s="79" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="79" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" s="79"/>
+      <c r="C2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="F2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="G2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="H2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="I2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="J2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="K2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="L2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="M2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="N2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="O2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="P2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="Q2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="R2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="S2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="T2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="U2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="V2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="W2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="X2" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="Y2" s="75" t="s">
+        <v>276</v>
+      </c>
+      <c r="Z2" s="75" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A3" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C3" s="76">
+        <v>136349</v>
+      </c>
+      <c r="D3" s="76">
+        <v>50.701683299999999</v>
+      </c>
+      <c r="E3" s="76">
+        <v>88893</v>
+      </c>
+      <c r="F3" s="76">
+        <v>71.660762700000006</v>
+      </c>
+      <c r="G3" s="76">
+        <v>89834</v>
+      </c>
+      <c r="H3" s="76">
+        <v>71.484235200000001</v>
+      </c>
+      <c r="I3" s="76">
+        <v>177063</v>
+      </c>
+      <c r="J3" s="76">
+        <v>25.208845199999999</v>
+      </c>
+      <c r="K3" s="76">
+        <v>105514</v>
+      </c>
+      <c r="L3" s="76">
+        <v>65.308434300000002</v>
+      </c>
+      <c r="M3" s="76">
+        <v>78825</v>
+      </c>
+      <c r="N3" s="76">
+        <v>75.404888099999994</v>
+      </c>
+      <c r="O3" s="76">
+        <v>74445</v>
+      </c>
+      <c r="P3" s="76">
+        <v>76.932256899999999</v>
+      </c>
+      <c r="Q3" s="76">
+        <v>154010</v>
+      </c>
+      <c r="R3" s="76">
+        <v>40.682205400000001</v>
+      </c>
+      <c r="S3" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T3" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U3" s="76">
+        <v>133274</v>
+      </c>
+      <c r="V3" s="76">
+        <v>52.362232400000003</v>
+      </c>
+      <c r="W3" s="76">
+        <v>56003</v>
+      </c>
+      <c r="X3" s="76">
+        <v>83.106039499999994</v>
+      </c>
+      <c r="Y3" s="76">
+        <v>171796</v>
+      </c>
+      <c r="Z3" s="76">
+        <v>28.984931</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A4" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C4" s="76">
+        <v>147689</v>
+      </c>
+      <c r="D4" s="76">
+        <v>44.259977499999998</v>
+      </c>
+      <c r="E4" s="76">
+        <v>153830</v>
+      </c>
+      <c r="F4" s="76">
+        <v>40.682205400000001</v>
+      </c>
+      <c r="G4" s="76">
+        <v>92076</v>
+      </c>
+      <c r="H4" s="76">
+        <v>70.618928299999993</v>
+      </c>
+      <c r="I4" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J4" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K4" s="76">
+        <v>97410</v>
+      </c>
+      <c r="L4" s="76">
+        <v>68.470259100000007</v>
+      </c>
+      <c r="M4" s="76">
+        <v>85698</v>
+      </c>
+      <c r="N4" s="76">
+        <v>73.134796199999997</v>
+      </c>
+      <c r="O4" s="76">
+        <v>78612</v>
+      </c>
+      <c r="P4" s="76">
+        <v>75.404888099999994</v>
+      </c>
+      <c r="Q4" s="76">
+        <v>160408</v>
+      </c>
+      <c r="R4" s="76">
+        <v>36.226011999999997</v>
+      </c>
+      <c r="S4" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T4" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U4" s="76">
+        <v>133274</v>
+      </c>
+      <c r="V4" s="76">
+        <v>52.362232400000003</v>
+      </c>
+      <c r="W4" s="76">
+        <v>56003</v>
+      </c>
+      <c r="X4" s="76">
+        <v>83.106039499999994</v>
+      </c>
+      <c r="Y4" s="76">
+        <v>171796</v>
+      </c>
+      <c r="Z4" s="76">
+        <v>28.984931</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A5" s="79" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C5" s="76">
+        <v>79469</v>
+      </c>
+      <c r="D5" s="76">
+        <v>75.210728000000003</v>
+      </c>
+      <c r="E5" s="76">
+        <v>55474</v>
+      </c>
+      <c r="F5" s="76">
+        <v>83.339724599999997</v>
+      </c>
+      <c r="G5" s="76">
+        <v>44738</v>
+      </c>
+      <c r="H5" s="76">
+        <v>86.675962999999996</v>
+      </c>
+      <c r="I5" s="76">
+        <v>74119</v>
+      </c>
+      <c r="J5" s="76">
+        <v>77.014977400000006</v>
+      </c>
+      <c r="K5" s="76">
+        <v>52268</v>
+      </c>
+      <c r="L5" s="76">
+        <v>84.329619500000007</v>
+      </c>
+      <c r="M5" s="76">
+        <v>46453</v>
+      </c>
+      <c r="N5" s="76">
+        <v>86.204101800000004</v>
+      </c>
+      <c r="O5" s="76">
+        <v>43336</v>
+      </c>
+      <c r="P5" s="76">
+        <v>87.137647799999996</v>
+      </c>
+      <c r="Q5" s="76">
+        <v>92865</v>
+      </c>
+      <c r="R5" s="76">
+        <v>70.500506400000006</v>
+      </c>
+      <c r="S5" s="76">
+        <v>108416</v>
+      </c>
+      <c r="T5" s="76">
+        <v>63.651287099999998</v>
+      </c>
+      <c r="U5" s="76">
+        <v>59819</v>
+      </c>
+      <c r="V5" s="76">
+        <v>81.940403000000003</v>
+      </c>
+      <c r="W5" s="76">
+        <v>32568</v>
+      </c>
+      <c r="X5" s="76">
+        <v>90.4253432</v>
+      </c>
+      <c r="Y5" s="76">
+        <v>89669</v>
+      </c>
+      <c r="Z5" s="76">
+        <v>71.556280799999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A6" s="79" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C6" s="76">
+        <v>71097</v>
+      </c>
+      <c r="D6" s="76">
+        <v>78.335764400000002</v>
+      </c>
+      <c r="E6" s="76">
+        <v>40771</v>
+      </c>
+      <c r="F6" s="76">
+        <v>87.928909399999995</v>
+      </c>
+      <c r="G6" s="76">
+        <v>39865</v>
+      </c>
+      <c r="H6" s="76">
+        <v>88.188033000000004</v>
+      </c>
+      <c r="I6" s="76">
+        <v>65789</v>
+      </c>
+      <c r="J6" s="76">
+        <v>79.907202699999999</v>
+      </c>
+      <c r="K6" s="76">
+        <v>38717</v>
+      </c>
+      <c r="L6" s="76">
+        <v>88.557388599999996</v>
+      </c>
+      <c r="M6" s="76">
+        <v>31233</v>
+      </c>
+      <c r="N6" s="76">
+        <v>90.873990899999995</v>
+      </c>
+      <c r="O6" s="76">
+        <v>42276</v>
+      </c>
+      <c r="P6" s="76">
+        <v>87.411539099999999</v>
+      </c>
+      <c r="Q6" s="76">
+        <v>82901</v>
+      </c>
+      <c r="R6" s="76">
+        <v>73.748251699999997</v>
+      </c>
+      <c r="S6" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T6" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U6" s="76">
+        <v>59819</v>
+      </c>
+      <c r="V6" s="76">
+        <v>81.940403000000003</v>
+      </c>
+      <c r="W6" s="76">
+        <v>32568</v>
+      </c>
+      <c r="X6" s="76">
+        <v>90.4253432</v>
+      </c>
+      <c r="Y6" s="76">
+        <v>89669</v>
+      </c>
+      <c r="Z6" s="76">
+        <v>71.556280799999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A7" s="79" t="s">
+        <v>289</v>
+      </c>
+      <c r="B7" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C7" s="76">
+        <v>87088</v>
+      </c>
+      <c r="D7" s="76">
+        <v>72.376095800000002</v>
+      </c>
+      <c r="E7" s="76">
+        <v>93475</v>
+      </c>
+      <c r="F7" s="76">
+        <v>70.203356700000001</v>
+      </c>
+      <c r="G7" s="76">
+        <v>71291</v>
+      </c>
+      <c r="H7" s="76">
+        <v>78.272232000000002</v>
+      </c>
+      <c r="I7" s="76">
+        <v>95795</v>
+      </c>
+      <c r="J7" s="76">
+        <v>69.097902099999999</v>
+      </c>
+      <c r="K7" s="76">
+        <v>81961</v>
+      </c>
+      <c r="L7" s="76">
+        <v>74.063078500000003</v>
+      </c>
+      <c r="M7" s="76">
+        <v>69461</v>
+      </c>
+      <c r="N7" s="76">
+        <v>78.613714799999997</v>
+      </c>
+      <c r="O7" s="76">
+        <v>66597</v>
+      </c>
+      <c r="P7" s="76">
+        <v>79.718500300000002</v>
+      </c>
+      <c r="Q7" s="76">
+        <v>152802</v>
+      </c>
+      <c r="R7" s="76">
+        <v>41.747128099999998</v>
+      </c>
+      <c r="S7" s="76">
+        <v>143884</v>
+      </c>
+      <c r="T7" s="76">
+        <v>47.0502678</v>
+      </c>
+      <c r="U7" s="76">
+        <v>185749</v>
+      </c>
+      <c r="V7" s="76">
+        <v>18.5475444</v>
+      </c>
+      <c r="W7" s="76">
+        <v>48232</v>
+      </c>
+      <c r="X7" s="76">
+        <v>85.618256400000007</v>
+      </c>
+      <c r="Y7" s="76">
+        <v>146092</v>
+      </c>
+      <c r="Z7" s="76">
+        <v>45.826605800000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A8" s="79" t="s">
+        <v>289</v>
+      </c>
+      <c r="B8" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C8" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="D8" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="E8" s="76">
+        <v>145990</v>
+      </c>
+      <c r="F8" s="76">
+        <v>45.826605800000003</v>
+      </c>
+      <c r="G8" s="76">
+        <v>79357</v>
+      </c>
+      <c r="H8" s="76">
+        <v>75.240591899999998</v>
+      </c>
+      <c r="I8" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J8" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K8" s="76">
+        <v>79445</v>
+      </c>
+      <c r="L8" s="76">
+        <v>75.240591899999998</v>
+      </c>
+      <c r="M8" s="76">
+        <v>67797</v>
+      </c>
+      <c r="N8" s="76">
+        <v>79.373089199999995</v>
+      </c>
+      <c r="O8" s="76">
+        <v>66347</v>
+      </c>
+      <c r="P8" s="76">
+        <v>79.794628200000005</v>
+      </c>
+      <c r="Q8" s="76">
+        <v>142436</v>
+      </c>
+      <c r="R8" s="76">
+        <v>47.356321800000003</v>
+      </c>
+      <c r="S8" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T8" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U8" s="76">
+        <v>185749</v>
+      </c>
+      <c r="V8" s="76">
+        <v>18.5475444</v>
+      </c>
+      <c r="W8" s="76">
+        <v>48232</v>
+      </c>
+      <c r="X8" s="76">
+        <v>85.618256400000007</v>
+      </c>
+      <c r="Y8" s="76">
+        <v>146092</v>
+      </c>
+      <c r="Z8" s="76">
+        <v>45.826605800000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A9" s="79" t="s">
+        <v>290</v>
+      </c>
+      <c r="B9" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C9" s="76">
+        <v>130622</v>
+      </c>
+      <c r="D9" s="76">
+        <v>53.759178200000001</v>
+      </c>
+      <c r="E9" s="76">
+        <v>103217</v>
+      </c>
+      <c r="F9" s="76">
+        <v>66.169536500000007</v>
+      </c>
+      <c r="G9" s="76">
+        <v>82903</v>
+      </c>
+      <c r="H9" s="76">
+        <v>73.748251699999997</v>
+      </c>
+      <c r="I9" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J9" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K9" s="77">
+        <v>92073</v>
+      </c>
+      <c r="L9" s="77">
+        <v>70.618928299999993</v>
+      </c>
+      <c r="M9" s="77">
+        <v>74421</v>
+      </c>
+      <c r="N9" s="77">
+        <v>76.932256899999999</v>
+      </c>
+      <c r="O9" s="77">
+        <v>72269</v>
+      </c>
+      <c r="P9" s="77">
+        <v>77.9513058</v>
+      </c>
+      <c r="Q9" s="77">
+        <v>138181</v>
+      </c>
+      <c r="R9" s="77">
+        <v>49.729110200000001</v>
+      </c>
+      <c r="S9" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T9" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U9" s="76">
+        <v>128352</v>
+      </c>
+      <c r="V9" s="76">
+        <v>54.587251799999997</v>
+      </c>
+      <c r="W9" s="76">
+        <v>56343</v>
+      </c>
+      <c r="X9" s="76">
+        <v>82.971748500000004</v>
+      </c>
+      <c r="Y9" s="76">
+        <v>146497</v>
+      </c>
+      <c r="Z9" s="76">
+        <v>45.356643400000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A10" s="79" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C10" s="76">
+        <v>107008</v>
+      </c>
+      <c r="D10" s="76">
+        <v>64.387101900000005</v>
+      </c>
+      <c r="E10" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="F10" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="G10" s="76">
+        <v>72183</v>
+      </c>
+      <c r="H10" s="76">
+        <v>78.010417000000004</v>
+      </c>
+      <c r="I10" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J10" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K10" s="77">
+        <v>75293</v>
+      </c>
+      <c r="L10" s="77">
+        <v>76.895550900000003</v>
+      </c>
+      <c r="M10" s="77">
+        <v>73248</v>
+      </c>
+      <c r="N10" s="77">
+        <v>77.163156599999994</v>
+      </c>
+      <c r="O10" s="77">
+        <v>59654</v>
+      </c>
+      <c r="P10" s="77">
+        <v>81.970591299999995</v>
+      </c>
+      <c r="Q10" s="77">
+        <v>126506</v>
+      </c>
+      <c r="R10" s="77">
+        <v>55.640575599999998</v>
+      </c>
+      <c r="S10" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T10" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U10" s="76">
+        <v>128352</v>
+      </c>
+      <c r="V10" s="76">
+        <v>54.587251799999997</v>
+      </c>
+      <c r="W10" s="76">
+        <v>56343</v>
+      </c>
+      <c r="X10" s="76">
+        <v>82.971748500000004</v>
+      </c>
+      <c r="Y10" s="76">
+        <v>146497</v>
+      </c>
+      <c r="Z10" s="76">
+        <v>45.356643400000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A11" s="79" t="s">
+        <v>291</v>
+      </c>
+      <c r="B11" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C11" s="78">
+        <v>95580</v>
+      </c>
+      <c r="D11" s="78">
+        <v>69.2179237</v>
+      </c>
+      <c r="E11" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="F11" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="G11" s="78">
+        <v>60001</v>
+      </c>
+      <c r="H11" s="78">
+        <v>81.802120099999996</v>
+      </c>
+      <c r="I11" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="J11" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="K11" s="78">
+        <v>66756</v>
+      </c>
+      <c r="L11" s="78">
+        <v>79.698602899999997</v>
+      </c>
+      <c r="M11" s="78">
+        <v>56492</v>
+      </c>
+      <c r="N11" s="78">
+        <v>82.971748500000004</v>
+      </c>
+      <c r="O11" s="78">
+        <v>56189</v>
+      </c>
+      <c r="P11" s="78">
+        <v>83.070771100000002</v>
+      </c>
+      <c r="Q11" s="78">
+        <v>106378</v>
+      </c>
+      <c r="R11" s="78">
+        <v>64.713185999999993</v>
+      </c>
+      <c r="S11" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="T11" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="U11" s="78">
+        <v>90759</v>
+      </c>
+      <c r="V11" s="78">
+        <v>71.173086999999995</v>
+      </c>
+      <c r="W11" s="78">
+        <v>53725</v>
+      </c>
+      <c r="X11" s="78">
+        <v>83.880236999999994</v>
+      </c>
+      <c r="Y11" s="78">
+        <v>133083</v>
+      </c>
+      <c r="Z11" s="78">
+        <v>52.596835599999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A12" s="79" t="s">
+        <v>291</v>
+      </c>
+      <c r="B12" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C12" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="D12" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="E12" s="78">
+        <v>117843</v>
+      </c>
+      <c r="F12" s="78">
+        <v>59.960701899999997</v>
+      </c>
+      <c r="G12" s="78">
+        <v>68091</v>
+      </c>
+      <c r="H12" s="78">
+        <v>79.300472600000006</v>
+      </c>
+      <c r="I12" s="78">
+        <v>153298</v>
+      </c>
+      <c r="J12" s="78">
+        <v>41.445818600000003</v>
+      </c>
+      <c r="K12" s="78">
+        <v>62938</v>
+      </c>
+      <c r="L12" s="78">
+        <v>81.013353499999994</v>
+      </c>
+      <c r="M12" s="78">
+        <v>51263</v>
+      </c>
+      <c r="N12" s="78">
+        <v>84.642981500000005</v>
+      </c>
+      <c r="O12" s="78">
+        <v>51209</v>
+      </c>
+      <c r="P12" s="78">
+        <v>84.642981500000005</v>
+      </c>
+      <c r="Q12" s="78">
+        <v>97656</v>
+      </c>
+      <c r="R12" s="78">
+        <v>68.470259100000007</v>
+      </c>
+      <c r="S12" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="T12" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="U12" s="78">
+        <v>90759</v>
+      </c>
+      <c r="V12" s="78">
+        <v>71.173086999999995</v>
+      </c>
+      <c r="W12" s="78">
+        <v>53725</v>
+      </c>
+      <c r="X12" s="78">
+        <v>83.880236999999994</v>
+      </c>
+      <c r="Y12" s="78">
+        <v>133083</v>
+      </c>
+      <c r="Z12" s="78">
+        <v>52.596835599999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A13" s="79" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C13" s="76">
+        <v>196375</v>
+      </c>
+      <c r="D13" s="76">
+        <v>8.7118702999999993</v>
+      </c>
+      <c r="E13" s="76">
+        <v>77682</v>
+      </c>
+      <c r="F13" s="76">
+        <v>75.652265</v>
+      </c>
+      <c r="G13" s="76">
+        <v>96992</v>
+      </c>
+      <c r="H13" s="76">
+        <v>68.868746700000003</v>
+      </c>
+      <c r="I13" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J13" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K13" s="76">
+        <v>109378</v>
+      </c>
+      <c r="L13" s="76">
+        <v>63.471422199999999</v>
+      </c>
+      <c r="M13" s="76">
+        <v>81919</v>
+      </c>
+      <c r="N13" s="76">
+        <v>74.063078500000003</v>
+      </c>
+      <c r="O13" s="76">
+        <v>76793</v>
+      </c>
+      <c r="P13" s="76">
+        <v>76.271685899999994</v>
+      </c>
+      <c r="Q13" s="76">
+        <v>130131</v>
+      </c>
+      <c r="R13" s="76">
+        <v>54.0903901</v>
+      </c>
+      <c r="S13" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T13" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U13" s="76">
+        <v>92532</v>
+      </c>
+      <c r="V13" s="76">
+        <v>70.500506400000006</v>
+      </c>
+      <c r="W13" s="76">
+        <v>63613</v>
+      </c>
+      <c r="X13" s="76">
+        <v>80.7175218</v>
+      </c>
+      <c r="Y13" s="76">
+        <v>197585</v>
+      </c>
+      <c r="Z13" s="76">
+        <v>7.4355244999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A14" s="79" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C14" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="D14" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="E14" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="F14" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="G14" s="76">
+        <v>111649</v>
+      </c>
+      <c r="H14" s="76">
+        <v>62.8632493</v>
+      </c>
+      <c r="I14" s="76">
+        <v>112233</v>
+      </c>
+      <c r="J14" s="76">
+        <v>62.136555600000001</v>
+      </c>
+      <c r="K14" s="76">
+        <v>88469</v>
+      </c>
+      <c r="L14" s="76">
+        <v>71.819719500000005</v>
+      </c>
+      <c r="M14" s="76">
+        <v>82331</v>
+      </c>
+      <c r="N14" s="76">
+        <v>74.009497199999998</v>
+      </c>
+      <c r="O14" s="76">
+        <v>67042</v>
+      </c>
+      <c r="P14" s="76">
+        <v>79.692509200000003</v>
+      </c>
+      <c r="Q14" s="76">
+        <v>161171</v>
+      </c>
+      <c r="R14" s="76">
+        <v>36.116164900000001</v>
+      </c>
+      <c r="S14" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T14" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U14" s="76">
+        <v>92532</v>
+      </c>
+      <c r="V14" s="76">
+        <v>70.500506400000006</v>
+      </c>
+      <c r="W14" s="76">
+        <v>63613</v>
+      </c>
+      <c r="X14" s="76">
+        <v>80.7175218</v>
+      </c>
+      <c r="Y14" s="76">
+        <v>197585</v>
+      </c>
+      <c r="Z14" s="76">
+        <v>7.4355244999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A15" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C15" s="76">
+        <v>55971</v>
+      </c>
+      <c r="D15" s="76">
+        <v>83.106039499999994</v>
+      </c>
+      <c r="E15" s="76">
+        <v>46780</v>
+      </c>
+      <c r="F15" s="76">
+        <v>85.977536000000001</v>
+      </c>
+      <c r="G15" s="76">
+        <v>44934</v>
+      </c>
+      <c r="H15" s="76">
+        <v>86.675175100000004</v>
+      </c>
+      <c r="I15" s="76">
+        <v>85022</v>
+      </c>
+      <c r="J15" s="76">
+        <v>73.435437899999997</v>
+      </c>
+      <c r="K15" s="76">
+        <v>109378</v>
+      </c>
+      <c r="L15" s="76">
+        <v>63.471422199999999</v>
+      </c>
+      <c r="M15" s="76">
+        <v>81919</v>
+      </c>
+      <c r="N15" s="76">
+        <v>74.063078500000003</v>
+      </c>
+      <c r="O15" s="76">
+        <v>76793</v>
+      </c>
+      <c r="P15" s="76">
+        <v>76.271685899999994</v>
+      </c>
+      <c r="Q15" s="76">
+        <v>130131</v>
+      </c>
+      <c r="R15" s="76">
+        <v>54.0903901</v>
+      </c>
+      <c r="S15" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T15" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U15" s="76">
+        <v>92481</v>
+      </c>
+      <c r="V15" s="76">
+        <v>70.507200999999995</v>
+      </c>
+      <c r="W15" s="76">
+        <v>29771</v>
+      </c>
+      <c r="X15" s="76">
+        <v>91.301571499999994</v>
+      </c>
+      <c r="Y15" s="76">
+        <v>91934</v>
+      </c>
+      <c r="Z15" s="76">
+        <v>70.618928299999993</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A16" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="B16" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C16" s="76">
+        <v>52646</v>
+      </c>
+      <c r="D16" s="76">
+        <v>84.143771599999994</v>
+      </c>
+      <c r="E16" s="76">
+        <v>40926</v>
+      </c>
+      <c r="F16" s="76">
+        <v>87.923517899999993</v>
+      </c>
+      <c r="G16" s="76">
+        <v>35113</v>
+      </c>
+      <c r="H16" s="76">
+        <v>89.682715000000002</v>
+      </c>
+      <c r="I16" s="76">
+        <v>77048</v>
+      </c>
+      <c r="J16" s="76">
+        <v>75.800195700000003</v>
+      </c>
+      <c r="K16" s="76">
+        <v>88469</v>
+      </c>
+      <c r="L16" s="76">
+        <v>71.819719500000005</v>
+      </c>
+      <c r="M16" s="76">
+        <v>82331</v>
+      </c>
+      <c r="N16" s="76">
+        <v>74.009497199999998</v>
+      </c>
+      <c r="O16" s="76">
+        <v>67042</v>
+      </c>
+      <c r="P16" s="76">
+        <v>79.692509200000003</v>
+      </c>
+      <c r="Q16" s="76">
+        <v>161171</v>
+      </c>
+      <c r="R16" s="76">
+        <v>36.116164900000001</v>
+      </c>
+      <c r="S16" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T16" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U16" s="76">
+        <v>92481</v>
+      </c>
+      <c r="V16" s="76">
+        <v>70.507200999999995</v>
+      </c>
+      <c r="W16" s="76">
+        <v>29771</v>
+      </c>
+      <c r="X16" s="76">
+        <v>91.301571499999994</v>
+      </c>
+      <c r="Y16" s="76">
+        <v>91934</v>
+      </c>
+      <c r="Z16" s="76">
+        <v>70.618928299999993</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A17" s="79" t="s">
+        <v>292</v>
+      </c>
+      <c r="B17" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C17" s="76">
+        <v>108028</v>
+      </c>
+      <c r="D17" s="76">
+        <v>63.824451400000001</v>
+      </c>
+      <c r="E17" s="76">
+        <v>170237</v>
+      </c>
+      <c r="F17" s="76">
+        <v>29.805952699999999</v>
+      </c>
+      <c r="G17" s="76">
+        <v>88151</v>
+      </c>
+      <c r="H17" s="76">
+        <v>71.849884399999993</v>
+      </c>
+      <c r="I17" s="76">
+        <v>140613</v>
+      </c>
+      <c r="J17" s="76">
+        <v>48.558742700000003</v>
+      </c>
+      <c r="K17" s="76">
+        <v>101869</v>
+      </c>
+      <c r="L17" s="76">
+        <v>66.426332299999999</v>
+      </c>
+      <c r="M17" s="76">
+        <v>86325</v>
+      </c>
+      <c r="N17" s="76">
+        <v>72.742941799999997</v>
+      </c>
+      <c r="O17" s="76">
+        <v>83677</v>
+      </c>
+      <c r="P17" s="76">
+        <v>73.632853600000004</v>
+      </c>
+      <c r="Q17" s="76">
+        <v>144835</v>
+      </c>
+      <c r="R17" s="76">
+        <v>46.395769600000001</v>
+      </c>
+      <c r="S17" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T17" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U17" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="V17" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="W17" s="76">
+        <v>82151</v>
+      </c>
+      <c r="X17" s="76">
+        <v>74.009497199999998</v>
+      </c>
+      <c r="Y17" s="76">
+        <v>192045</v>
+      </c>
+      <c r="Z17" s="76">
+        <v>12.9554081</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A18" s="79" t="s">
+        <v>292</v>
+      </c>
+      <c r="B18" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="D18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="E18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="F18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="G18" s="76">
+        <v>123397</v>
+      </c>
+      <c r="H18" s="76">
+        <v>57.401745900000002</v>
+      </c>
+      <c r="I18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K18" s="76">
+        <v>93796</v>
+      </c>
+      <c r="L18" s="76">
+        <v>69.894105100000004</v>
+      </c>
+      <c r="M18" s="76">
+        <v>82886</v>
+      </c>
+      <c r="N18" s="76">
+        <v>73.748251699999997</v>
+      </c>
+      <c r="O18" s="76">
+        <v>69681</v>
+      </c>
+      <c r="P18" s="76">
+        <v>78.613714799999997</v>
+      </c>
+      <c r="Q18" s="76">
+        <v>87753</v>
+      </c>
+      <c r="R18" s="76">
+        <v>72.102801999999997</v>
+      </c>
+      <c r="S18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="V18" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="W18" s="76">
+        <v>82151</v>
+      </c>
+      <c r="X18" s="76">
+        <v>74.009497199999998</v>
+      </c>
+      <c r="Y18" s="76">
+        <v>192045</v>
+      </c>
+      <c r="Z18" s="76">
+        <v>12.9554081</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A19" s="79" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" s="75" t="s">
+        <v>273</v>
+      </c>
+      <c r="C19" s="76">
+        <v>111550</v>
+      </c>
+      <c r="D19" s="76">
+        <v>65.669275099999993</v>
+      </c>
+      <c r="E19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="F19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="G19" s="76">
+        <v>44154</v>
+      </c>
+      <c r="H19" s="76">
+        <v>87.898058000000006</v>
+      </c>
+      <c r="I19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K19" s="76">
+        <v>49375</v>
+      </c>
+      <c r="L19" s="76">
+        <v>86.344100900000001</v>
+      </c>
+      <c r="M19" s="76">
+        <v>40077</v>
+      </c>
+      <c r="N19" s="76">
+        <v>88.977569799999998</v>
+      </c>
+      <c r="O19" s="76">
+        <v>38139</v>
+      </c>
+      <c r="P19" s="76">
+        <v>89.535526200000007</v>
+      </c>
+      <c r="Q19" s="76">
+        <v>86462</v>
+      </c>
+      <c r="R19" s="76">
+        <v>75.096259599999996</v>
+      </c>
+      <c r="S19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="V19" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="W19" s="76">
+        <v>17985</v>
+      </c>
+      <c r="X19" s="76">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="76">
+        <v>126918</v>
+      </c>
+      <c r="Z19" s="76">
+        <v>59.097417900000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A20" s="79" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="C20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="D20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="E20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="F20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="G20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="H20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="I20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="J20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="K20" s="76">
+        <v>43083</v>
+      </c>
+      <c r="L20" s="76">
+        <v>88.132563300000001</v>
+      </c>
+      <c r="M20" s="76">
+        <v>25616</v>
+      </c>
+      <c r="N20" s="76">
+        <v>93.077884999999995</v>
+      </c>
+      <c r="O20" s="76">
+        <v>24721</v>
+      </c>
+      <c r="P20" s="76">
+        <v>93.282577399999994</v>
+      </c>
+      <c r="Q20" s="76">
+        <v>59582</v>
+      </c>
+      <c r="R20" s="76">
+        <v>83.255577599999995</v>
+      </c>
+      <c r="S20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="T20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="U20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="V20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="W20" s="76">
+        <v>17985</v>
+      </c>
+      <c r="X20" s="76">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="76">
+        <v>126918</v>
+      </c>
+      <c r="Z20" s="76">
+        <v>59.097417900000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>